<commit_message>
Site_Definition_Cleanup: remove Actuator Type column from Dehydrators (issue #38)
Arthur clarified it should be excluded, not kept.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/Studies/MEET2/AllEquipment.xlsx
+++ b/input/Studies/MEET2/AllEquipment.xlsx
@@ -5967,7 +5967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5992,75 +5992,70 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Actuator Type [Gas, Electric, Air]</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
           <t>Model ID</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Flash Tank</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Flash Tank</t>
+          <t>Glycol Pump</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Glycol Pump</t>
+          <t>Glycol Pump Injection Ratio</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Glycol Pump Injection Ratio</t>
+          <t>Glycol Type</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Glycol Type</t>
+          <t>Lean Glycol Circulation Rate</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Lean Glycol Circulation Rate</t>
+          <t>Lean Glycol Circulation Ratio</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Lean Glycol Circulation Ratio</t>
+          <t>Operating Hours</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Operating Hours</t>
+          <t>Still Vent Controlled Flag</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Still Vent Controlled Flag</t>
+          <t>Stripping Gas Flow Rate</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Stripping Gas Flow Rate</t>
+          <t>Tank Flash Controlled Flag</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Tank Flash Controlled Flag</t>
+          <t>Wet Gas Flow Rate</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Wet Gas Flow Rate</t>
+          <t>Wet Gas Pressure</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
-        <is>
-          <t>Wet Gas Pressure</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
         <is>
           <t>Wet Gas Temperature</t>
         </is>
@@ -6077,57 +6072,52 @@
           <t>dehy_1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Gas</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Dehydrator.json</t>
         </is>
       </c>
-      <c r="E2" t="b">
+      <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Gas Assisted</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="F2" t="n">
         <v>4.5</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>TEG</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J2" t="n">
+        <v>8760</v>
+      </c>
+      <c r="K2" t="b">
         <v>0</v>
       </c>
-      <c r="J2" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="K2" t="n">
-        <v>8760</v>
-      </c>
-      <c r="L2" t="b">
+      <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" t="b">
         <v>0</v>
       </c>
-      <c r="N2" t="b">
-        <v>0</v>
+      <c r="N2" t="n">
+        <v>100000</v>
       </c>
       <c r="O2" t="n">
-        <v>100000</v>
+        <v>957</v>
       </c>
       <c r="P2" t="n">
-        <v>957</v>
-      </c>
-      <c r="Q2" t="n">
         <v>92.40000000000001</v>
       </c>
     </row>

</xml_diff>